<commit_message>
fix: corrigir extração de dados — remover duplicatas e melhorar OCR
- CartaoPontoExtractor: filtrar datas de cabeçalho/rodapé repetidas em
  múltiplas páginas (removeRepeatedHeaderDates com threshold >= 3 páginas)
- HoleriteExtractor: mesclar entradas duplicadas do mesmo mês/página na
  Ficha Financeira quando campos se sobrepõem (mergeDuplicateEntries)
- PDF_RENDER_SCALE: 4 → 5 (~288 DPI → ~360 DPI, mais próximo de 300)
- OCR_CONFIDENCE_THRESHOLD: 40 → 60 (mais restritivo)
- Atualizar samples, CHANGELOG, SOLUCAO e .env.example
- Versão 1.2.0 → 1.3.0
</commit_message>
<xml_diff>
--- a/exemplos/output/payroll-01.xlsx
+++ b/exemplos/output/payroll-01.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1566" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1296" uniqueCount="261">
   <si>
     <t>Pág.</t>
   </si>
@@ -355,36 +355,36 @@
     <t>10</t>
   </si>
   <si>
+    <t>1.567,25</t>
+  </si>
+  <si>
+    <t>50,14</t>
+  </si>
+  <si>
+    <t>2,58</t>
+  </si>
+  <si>
+    <t>470,18</t>
+  </si>
+  <si>
+    <t>190,14</t>
+  </si>
+  <si>
+    <t>94,04</t>
+  </si>
+  <si>
+    <t>3,45</t>
+  </si>
+  <si>
+    <t>13,82</t>
+  </si>
+  <si>
+    <t>1,39</t>
+  </si>
+  <si>
     <t>2.819,91</t>
   </si>
   <si>
-    <t>1.567,25</t>
-  </si>
-  <si>
-    <t>50,14</t>
-  </si>
-  <si>
-    <t>2,58</t>
-  </si>
-  <si>
-    <t>470,18</t>
-  </si>
-  <si>
-    <t>190,14</t>
-  </si>
-  <si>
-    <t>94,04</t>
-  </si>
-  <si>
-    <t>3,45</t>
-  </si>
-  <si>
-    <t>13,82</t>
-  </si>
-  <si>
-    <t>1,39</t>
-  </si>
-  <si>
     <t>59,45</t>
   </si>
   <si>
@@ -445,81 +445,81 @@
     <t>173,38</t>
   </si>
   <si>
+    <t>1.692,42</t>
+  </si>
+  <si>
     <t>6,21</t>
   </si>
   <si>
+    <t>349,11</t>
+  </si>
+  <si>
+    <t>31,96</t>
+  </si>
+  <si>
+    <t>97,78</t>
+  </si>
+  <si>
+    <t>3,51</t>
+  </si>
+  <si>
+    <t>1.528,07</t>
+  </si>
+  <si>
+    <t>200,83</t>
+  </si>
+  <si>
+    <t>749,19</t>
+  </si>
+  <si>
+    <t>3.714,04</t>
+  </si>
+  <si>
+    <t>72,55</t>
+  </si>
+  <si>
+    <t>160,23</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>02</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>193,52</t>
+  </si>
+  <si>
+    <t>18,81</t>
+  </si>
+  <si>
+    <t>94,09</t>
+  </si>
+  <si>
+    <t>458,42</t>
+  </si>
+  <si>
+    <t>03</t>
+  </si>
+  <si>
+    <t>69,30</t>
+  </si>
+  <si>
+    <t>216,38</t>
+  </si>
+  <si>
+    <t>61,15</t>
+  </si>
+  <si>
+    <t>150,15</t>
+  </si>
+  <si>
     <t>155,60</t>
   </si>
   <si>
-    <t>31,96</t>
-  </si>
-  <si>
-    <t>3,51</t>
-  </si>
-  <si>
-    <t>1.528,07</t>
-  </si>
-  <si>
-    <t>200,83</t>
-  </si>
-  <si>
-    <t>749,19</t>
-  </si>
-  <si>
-    <t>1.692,42</t>
-  </si>
-  <si>
-    <t>349,11</t>
-  </si>
-  <si>
-    <t>97,78</t>
-  </si>
-  <si>
-    <t>3.714,04</t>
-  </si>
-  <si>
-    <t>72,55</t>
-  </si>
-  <si>
-    <t>160,23</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>02</t>
-  </si>
-  <si>
-    <t>2018</t>
-  </si>
-  <si>
-    <t>458,42</t>
-  </si>
-  <si>
-    <t>193,52</t>
-  </si>
-  <si>
-    <t>18,81</t>
-  </si>
-  <si>
-    <t>94,09</t>
-  </si>
-  <si>
-    <t>03</t>
-  </si>
-  <si>
-    <t>69,30</t>
-  </si>
-  <si>
-    <t>216,38</t>
-  </si>
-  <si>
-    <t>61,15</t>
-  </si>
-  <si>
-    <t>150,15</t>
-  </si>
-  <si>
     <t>212,46</t>
   </si>
   <si>
@@ -643,42 +643,42 @@
     <t>713,23</t>
   </si>
   <si>
+    <t>1.516,01</t>
+  </si>
+  <si>
+    <t>205,33</t>
+  </si>
+  <si>
+    <t>1,82</t>
+  </si>
+  <si>
+    <t>454,80</t>
+  </si>
+  <si>
+    <t>228,93</t>
+  </si>
+  <si>
+    <t>90,96</t>
+  </si>
+  <si>
+    <t>762,39</t>
+  </si>
+  <si>
+    <t>43,72</t>
+  </si>
+  <si>
+    <t>91,64</t>
+  </si>
+  <si>
+    <t>126,98</t>
+  </si>
+  <si>
+    <t>4,48</t>
+  </si>
+  <si>
     <t>3.878,54</t>
   </si>
   <si>
-    <t>1.516,01</t>
-  </si>
-  <si>
-    <t>205,33</t>
-  </si>
-  <si>
-    <t>1,82</t>
-  </si>
-  <si>
-    <t>454,80</t>
-  </si>
-  <si>
-    <t>228,93</t>
-  </si>
-  <si>
-    <t>90,96</t>
-  </si>
-  <si>
-    <t>762,39</t>
-  </si>
-  <si>
-    <t>43,72</t>
-  </si>
-  <si>
-    <t>91,64</t>
-  </si>
-  <si>
-    <t>126,98</t>
-  </si>
-  <si>
-    <t>4,48</t>
-  </si>
-  <si>
     <t>3,80</t>
   </si>
   <si>
@@ -760,25 +760,25 @@
     <t>2019</t>
   </si>
   <si>
+    <t>50,00</t>
+  </si>
+  <si>
+    <t>65,55</t>
+  </si>
+  <si>
+    <t>216,59</t>
+  </si>
+  <si>
+    <t>49,17</t>
+  </si>
+  <si>
+    <t>120,31</t>
+  </si>
+  <si>
+    <t>125,55</t>
+  </si>
+  <si>
     <t>633,48</t>
-  </si>
-  <si>
-    <t>50,00</t>
-  </si>
-  <si>
-    <t>65,55</t>
-  </si>
-  <si>
-    <t>216,59</t>
-  </si>
-  <si>
-    <t>49,17</t>
-  </si>
-  <si>
-    <t>120,31</t>
-  </si>
-  <si>
-    <t>125,55</t>
   </si>
   <si>
     <t>79,35</t>
@@ -1195,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BB29"/>
+  <dimension ref="A1:BB24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="54" width="18" customWidth="1"/>
@@ -2360,73 +2360,73 @@
         <v>56</v>
       </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>114</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>115</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G8" t="s">
-        <v>67</v>
+        <v>116</v>
       </c>
       <c r="H8" t="s">
         <v>67</v>
       </c>
       <c r="I8" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="J8" t="s">
-        <v>67</v>
+        <v>117</v>
       </c>
       <c r="K8" t="s">
-        <v>67</v>
+        <v>118</v>
       </c>
       <c r="L8" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M8" t="s">
-        <v>67</v>
+        <v>119</v>
       </c>
       <c r="N8" t="s">
-        <v>67</v>
+        <v>108</v>
       </c>
       <c r="O8" t="s">
-        <v>67</v>
+        <v>120</v>
       </c>
       <c r="P8" t="s">
-        <v>67</v>
+        <v>121</v>
       </c>
       <c r="Q8" t="s">
         <v>67</v>
       </c>
       <c r="R8" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="S8" t="s">
-        <v>67</v>
+        <v>111</v>
       </c>
       <c r="T8" t="s">
-        <v>67</v>
+        <v>122</v>
       </c>
       <c r="U8" t="s">
         <v>67</v>
       </c>
       <c r="V8" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="W8" t="s">
         <v>65</v>
       </c>
       <c r="X8" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="Y8" t="s">
-        <v>67</v>
+        <v>123</v>
       </c>
       <c r="Z8" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
       <c r="AA8" t="s">
         <v>67</v>
@@ -2514,166 +2514,166 @@
       </c>
     </row>
     <row r="9" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="B9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E9" s="2" t="s">
+      <c r="D9" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G9" t="s">
         <v>116</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" t="s">
+        <v>127</v>
+      </c>
+      <c r="I9" t="s">
+        <v>128</v>
+      </c>
+      <c r="J9" t="s">
         <v>117</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K9" s="2" t="s">
+      <c r="K9" t="s">
+        <v>129</v>
+      </c>
+      <c r="L9" t="s">
+        <v>130</v>
+      </c>
+      <c r="M9" t="s">
         <v>119</v>
       </c>
-      <c r="L9" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="O9" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="S9" s="2" t="s">
+      <c r="N9" t="s">
+        <v>131</v>
+      </c>
+      <c r="O9" t="s">
+        <v>132</v>
+      </c>
+      <c r="P9" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>134</v>
+      </c>
+      <c r="R9" t="s">
+        <v>135</v>
+      </c>
+      <c r="S9" t="s">
         <v>111</v>
       </c>
-      <c r="T9" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="U9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V9" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="X9" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="Y9" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA9" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB9" s="2" t="s">
+      <c r="T9" t="s">
+        <v>67</v>
+      </c>
+      <c r="U9" t="s">
+        <v>67</v>
+      </c>
+      <c r="V9" t="s">
+        <v>67</v>
+      </c>
+      <c r="W9" t="s">
+        <v>67</v>
+      </c>
+      <c r="X9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB9" t="s">
+        <v>137</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>137</v>
+      </c>
+      <c r="AD9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AI9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AX9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AY9" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ9" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA9" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB9" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2682,13 +2682,13 @@
         <v>112</v>
       </c>
       <c r="B10" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="C10" t="s">
         <v>56</v>
       </c>
       <c r="D10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E10" t="s">
         <v>126</v>
@@ -2697,37 +2697,37 @@
         <v>71</v>
       </c>
       <c r="G10" t="s">
+        <v>116</v>
+      </c>
+      <c r="H10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" t="s">
         <v>117</v>
       </c>
-      <c r="H10" t="s">
-        <v>127</v>
-      </c>
-      <c r="I10" t="s">
-        <v>128</v>
-      </c>
-      <c r="J10" t="s">
-        <v>118</v>
-      </c>
       <c r="K10" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="L10" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="M10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N10" t="s">
         <v>131</v>
       </c>
       <c r="O10" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="P10" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="Q10" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="R10" t="s">
         <v>135</v>
@@ -2757,49 +2757,49 @@
         <v>67</v>
       </c>
       <c r="AA10" t="s">
-        <v>136</v>
+        <v>67</v>
       </c>
       <c r="AB10" t="s">
-        <v>137</v>
+        <v>67</v>
       </c>
       <c r="AC10" t="s">
-        <v>137</v>
+        <v>67</v>
       </c>
       <c r="AD10" t="s">
-        <v>67</v>
+        <v>144</v>
       </c>
       <c r="AE10" t="s">
-        <v>67</v>
+        <v>145</v>
       </c>
       <c r="AF10" t="s">
-        <v>67</v>
+        <v>146</v>
       </c>
       <c r="AG10" t="s">
-        <v>67</v>
+        <v>147</v>
       </c>
       <c r="AH10" t="s">
-        <v>67</v>
+        <v>148</v>
       </c>
       <c r="AI10" t="s">
-        <v>67</v>
+        <v>149</v>
       </c>
       <c r="AJ10" t="s">
-        <v>67</v>
+        <v>150</v>
       </c>
       <c r="AK10" t="s">
-        <v>67</v>
+        <v>151</v>
       </c>
       <c r="AL10" t="s">
-        <v>67</v>
+        <v>152</v>
       </c>
       <c r="AM10" t="s">
-        <v>67</v>
+        <v>153</v>
       </c>
       <c r="AN10" t="s">
-        <v>67</v>
+        <v>154</v>
       </c>
       <c r="AO10" t="s">
-        <v>67</v>
+        <v>155</v>
       </c>
       <c r="AP10" t="s">
         <v>67</v>
@@ -2842,673 +2842,673 @@
       </c>
     </row>
     <row r="11" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>112</v>
-      </c>
-      <c r="B11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C11" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" t="s">
-        <v>115</v>
-      </c>
-      <c r="E11" t="s">
+      <c r="A11" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="H11" t="s">
-        <v>72</v>
-      </c>
-      <c r="I11" t="s">
-        <v>72</v>
-      </c>
-      <c r="J11" t="s">
-        <v>118</v>
-      </c>
-      <c r="K11" t="s">
-        <v>139</v>
-      </c>
-      <c r="L11" t="s">
-        <v>140</v>
-      </c>
-      <c r="M11" t="s">
-        <v>120</v>
-      </c>
-      <c r="N11" t="s">
+      <c r="K11" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="O11" t="s">
-        <v>141</v>
-      </c>
-      <c r="P11" t="s">
-        <v>142</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>143</v>
-      </c>
-      <c r="R11" t="s">
+      <c r="O11" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="R11" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="S11" t="s">
+      <c r="S11" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="T11" t="s">
-        <v>67</v>
-      </c>
-      <c r="U11" t="s">
-        <v>67</v>
-      </c>
-      <c r="V11" t="s">
-        <v>67</v>
-      </c>
-      <c r="W11" t="s">
-        <v>67</v>
-      </c>
-      <c r="X11" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y11" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>137</v>
-      </c>
-      <c r="AE11" t="s">
-        <v>144</v>
-      </c>
-      <c r="AF11" t="s">
-        <v>145</v>
-      </c>
-      <c r="AG11" t="s">
-        <v>146</v>
-      </c>
-      <c r="AH11" t="s">
+      <c r="T11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="W11" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="AI11" t="s">
-        <v>147</v>
-      </c>
-      <c r="AJ11" t="s">
-        <v>148</v>
-      </c>
-      <c r="AK11" t="s">
-        <v>149</v>
-      </c>
-      <c r="AL11" t="s">
-        <v>150</v>
-      </c>
-      <c r="AM11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY11" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ11" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA11" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB11" t="s">
+      <c r="X11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y11" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="Z11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AI11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AX11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AY11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB11" s="2" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="O12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="P12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="S12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="W12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="X12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD12" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="AE12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF12" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="AG12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH12" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="AI12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM12" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="AN12" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="AO12" s="2" t="s">
+      <c r="A12" t="s">
         <v>156</v>
       </c>
-      <c r="AP12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA12" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB12" s="2" t="s">
+      <c r="B12" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D12" t="s">
+        <v>114</v>
+      </c>
+      <c r="E12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G12" t="s">
+        <v>116</v>
+      </c>
+      <c r="H12" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" t="s">
+        <v>164</v>
+      </c>
+      <c r="J12" t="s">
+        <v>117</v>
+      </c>
+      <c r="K12" t="s">
+        <v>165</v>
+      </c>
+      <c r="L12" t="s">
+        <v>65</v>
+      </c>
+      <c r="M12" t="s">
+        <v>119</v>
+      </c>
+      <c r="N12" t="s">
+        <v>131</v>
+      </c>
+      <c r="O12" t="s">
+        <v>166</v>
+      </c>
+      <c r="P12" t="s">
+        <v>167</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>168</v>
+      </c>
+      <c r="R12" t="s">
+        <v>135</v>
+      </c>
+      <c r="S12" t="s">
+        <v>111</v>
+      </c>
+      <c r="T12" t="s">
+        <v>67</v>
+      </c>
+      <c r="U12" t="s">
+        <v>67</v>
+      </c>
+      <c r="V12" t="s">
+        <v>67</v>
+      </c>
+      <c r="W12" t="s">
+        <v>67</v>
+      </c>
+      <c r="X12" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AI12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AX12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AY12" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ12" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA12" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB12" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A13" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="B13" s="2" t="s">
+      <c r="A13" t="s">
+        <v>156</v>
+      </c>
+      <c r="B13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" t="s">
         <v>158</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="P13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V13" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="W13" s="2" t="s">
+      <c r="D13" t="s">
+        <v>114</v>
+      </c>
+      <c r="E13" t="s">
+        <v>126</v>
+      </c>
+      <c r="F13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" t="s">
+        <v>116</v>
+      </c>
+      <c r="H13" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" t="s">
+        <v>164</v>
+      </c>
+      <c r="J13" t="s">
+        <v>117</v>
+      </c>
+      <c r="K13" t="s">
+        <v>169</v>
+      </c>
+      <c r="L13" t="s">
         <v>65</v>
       </c>
-      <c r="X13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA13" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB13" s="2" t="s">
+      <c r="M13" t="s">
+        <v>119</v>
+      </c>
+      <c r="N13" t="s">
+        <v>131</v>
+      </c>
+      <c r="O13" t="s">
+        <v>170</v>
+      </c>
+      <c r="P13" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>172</v>
+      </c>
+      <c r="R13" t="s">
+        <v>135</v>
+      </c>
+      <c r="S13" t="s">
+        <v>173</v>
+      </c>
+      <c r="T13" t="s">
+        <v>67</v>
+      </c>
+      <c r="U13" t="s">
+        <v>67</v>
+      </c>
+      <c r="V13" t="s">
+        <v>67</v>
+      </c>
+      <c r="W13" t="s">
+        <v>67</v>
+      </c>
+      <c r="X13" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AI13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AX13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AY13" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ13" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA13" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB13" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="B14" s="2" t="s">
+      <c r="A14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s">
         <v>158</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="E14" s="2" t="s">
+      <c r="D14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E14" t="s">
         <v>126</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" t="s">
         <v>71</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" t="s">
+        <v>116</v>
+      </c>
+      <c r="H14" t="s">
+        <v>174</v>
+      </c>
+      <c r="I14" t="s">
+        <v>164</v>
+      </c>
+      <c r="J14" t="s">
         <v>117</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="L14" s="2" t="s">
+      <c r="K14" t="s">
+        <v>175</v>
+      </c>
+      <c r="L14" t="s">
         <v>65</v>
       </c>
-      <c r="M14" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N14" s="2" t="s">
+      <c r="M14" t="s">
+        <v>176</v>
+      </c>
+      <c r="N14" t="s">
         <v>131</v>
       </c>
-      <c r="O14" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="P14" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="Q14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R14" s="2" t="s">
+      <c r="O14" t="s">
+        <v>177</v>
+      </c>
+      <c r="P14" t="s">
+        <v>178</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>179</v>
+      </c>
+      <c r="R14" t="s">
         <v>135</v>
       </c>
-      <c r="S14" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="T14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V14" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="W14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="X14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y14" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="Z14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA14" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB14" s="2" t="s">
+      <c r="S14" t="s">
+        <v>180</v>
+      </c>
+      <c r="T14" t="s">
+        <v>67</v>
+      </c>
+      <c r="U14" t="s">
+        <v>67</v>
+      </c>
+      <c r="V14" t="s">
+        <v>67</v>
+      </c>
+      <c r="W14" t="s">
+        <v>67</v>
+      </c>
+      <c r="X14" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y14" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AE14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AG14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AI14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AN14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AO14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AP14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AX14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AY14" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ14" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA14" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB14" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B15" t="s">
-        <v>164</v>
+        <v>81</v>
       </c>
       <c r="C15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
         <v>126</v>
@@ -3517,43 +3517,43 @@
         <v>71</v>
       </c>
       <c r="G15" t="s">
+        <v>116</v>
+      </c>
+      <c r="H15" t="s">
+        <v>67</v>
+      </c>
+      <c r="I15" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" t="s">
         <v>117</v>
       </c>
-      <c r="H15" t="s">
-        <v>127</v>
-      </c>
-      <c r="I15" t="s">
-        <v>165</v>
-      </c>
-      <c r="J15" t="s">
-        <v>118</v>
-      </c>
       <c r="K15" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="L15" t="s">
-        <v>65</v>
+        <v>182</v>
       </c>
       <c r="M15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N15" t="s">
         <v>131</v>
       </c>
       <c r="O15" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="P15" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
       <c r="Q15" t="s">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="R15" t="s">
         <v>135</v>
       </c>
       <c r="S15" t="s">
-        <v>111</v>
+        <v>180</v>
       </c>
       <c r="T15" t="s">
         <v>67</v>
@@ -3622,13 +3622,13 @@
         <v>67</v>
       </c>
       <c r="AP15" t="s">
-        <v>67</v>
+        <v>186</v>
       </c>
       <c r="AQ15" t="s">
-        <v>67</v>
+        <v>187</v>
       </c>
       <c r="AR15" t="s">
-        <v>67</v>
+        <v>188</v>
       </c>
       <c r="AS15" t="s">
         <v>67</v>
@@ -3663,61 +3663,61 @@
     </row>
     <row r="16" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>88</v>
       </c>
       <c r="C16" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E16" t="s">
         <v>126</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G16" t="s">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="H16" t="s">
-        <v>127</v>
+        <v>67</v>
       </c>
       <c r="I16" t="s">
-        <v>165</v>
+        <v>67</v>
       </c>
       <c r="J16" t="s">
-        <v>118</v>
+        <v>67</v>
       </c>
       <c r="K16" t="s">
-        <v>169</v>
+        <v>67</v>
       </c>
       <c r="L16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="M16" t="s">
-        <v>120</v>
+        <v>67</v>
       </c>
       <c r="N16" t="s">
-        <v>131</v>
+        <v>67</v>
       </c>
       <c r="O16" t="s">
-        <v>170</v>
+        <v>67</v>
       </c>
       <c r="P16" t="s">
-        <v>171</v>
+        <v>67</v>
       </c>
       <c r="Q16" t="s">
-        <v>172</v>
+        <v>67</v>
       </c>
       <c r="R16" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
       <c r="S16" t="s">
-        <v>173</v>
+        <v>67</v>
       </c>
       <c r="T16" t="s">
         <v>67</v>
@@ -3827,16 +3827,16 @@
     </row>
     <row r="17" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>157</v>
+        <v>189</v>
       </c>
       <c r="B17" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="C17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E17" t="s">
         <v>126</v>
@@ -3845,37 +3845,37 @@
         <v>71</v>
       </c>
       <c r="G17" t="s">
+        <v>190</v>
+      </c>
+      <c r="H17" t="s">
+        <v>191</v>
+      </c>
+      <c r="I17" t="s">
+        <v>192</v>
+      </c>
+      <c r="J17" t="s">
         <v>117</v>
       </c>
-      <c r="H17" t="s">
-        <v>174</v>
-      </c>
-      <c r="I17" t="s">
-        <v>165</v>
-      </c>
-      <c r="J17" t="s">
-        <v>118</v>
-      </c>
       <c r="K17" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="L17" t="s">
         <v>65</v>
       </c>
       <c r="M17" t="s">
-        <v>176</v>
+        <v>119</v>
       </c>
       <c r="N17" t="s">
         <v>131</v>
       </c>
       <c r="O17" t="s">
-        <v>177</v>
+        <v>194</v>
       </c>
       <c r="P17" t="s">
-        <v>178</v>
+        <v>195</v>
       </c>
       <c r="Q17" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="R17" t="s">
         <v>135</v>
@@ -3953,7 +3953,7 @@
         <v>67</v>
       </c>
       <c r="AQ17" t="s">
-        <v>67</v>
+        <v>187</v>
       </c>
       <c r="AR17" t="s">
         <v>67</v>
@@ -3991,55 +3991,55 @@
     </row>
     <row r="18" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>157</v>
+        <v>189</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="C18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D18" t="s">
-        <v>115</v>
+        <v>197</v>
       </c>
       <c r="E18" t="s">
         <v>126</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>198</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>190</v>
       </c>
       <c r="H18" t="s">
         <v>67</v>
       </c>
       <c r="I18" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="J18" t="s">
-        <v>118</v>
+        <v>199</v>
       </c>
       <c r="K18" t="s">
-        <v>181</v>
+        <v>200</v>
       </c>
       <c r="L18" t="s">
-        <v>182</v>
+        <v>67</v>
       </c>
       <c r="M18" t="s">
-        <v>120</v>
+        <v>67</v>
       </c>
       <c r="N18" t="s">
-        <v>131</v>
+        <v>67</v>
       </c>
       <c r="O18" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="P18" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="Q18" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
       <c r="R18" t="s">
         <v>135</v>
@@ -4072,7 +4072,7 @@
         <v>67</v>
       </c>
       <c r="AB18" t="s">
-        <v>67</v>
+        <v>204</v>
       </c>
       <c r="AC18" t="s">
         <v>67</v>
@@ -4114,28 +4114,28 @@
         <v>67</v>
       </c>
       <c r="AP18" t="s">
-        <v>186</v>
+        <v>67</v>
       </c>
       <c r="AQ18" t="s">
-        <v>187</v>
+        <v>67</v>
       </c>
       <c r="AR18" t="s">
-        <v>188</v>
+        <v>67</v>
       </c>
       <c r="AS18" t="s">
-        <v>67</v>
+        <v>205</v>
       </c>
       <c r="AT18" t="s">
-        <v>67</v>
+        <v>206</v>
       </c>
       <c r="AU18" t="s">
-        <v>67</v>
+        <v>207</v>
       </c>
       <c r="AV18" t="s">
-        <v>67</v>
+        <v>208</v>
       </c>
       <c r="AW18" t="s">
-        <v>67</v>
+        <v>209</v>
       </c>
       <c r="AX18" t="s">
         <v>67</v>
@@ -4155,61 +4155,61 @@
     </row>
     <row r="19" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>157</v>
+        <v>189</v>
       </c>
       <c r="B19" t="s">
-        <v>88</v>
+        <v>113</v>
       </c>
       <c r="C19" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D19" t="s">
-        <v>115</v>
+        <v>210</v>
       </c>
       <c r="E19" t="s">
         <v>126</v>
       </c>
       <c r="F19" t="s">
-        <v>67</v>
+        <v>211</v>
       </c>
       <c r="G19" t="s">
-        <v>67</v>
+        <v>212</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>127</v>
       </c>
       <c r="I19" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="J19" t="s">
-        <v>67</v>
+        <v>213</v>
       </c>
       <c r="K19" t="s">
-        <v>67</v>
+        <v>214</v>
       </c>
       <c r="L19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M19" t="s">
-        <v>67</v>
+        <v>215</v>
       </c>
       <c r="N19" t="s">
-        <v>67</v>
+        <v>216</v>
       </c>
       <c r="O19" t="s">
-        <v>67</v>
+        <v>217</v>
       </c>
       <c r="P19" t="s">
-        <v>67</v>
+        <v>218</v>
       </c>
       <c r="Q19" t="s">
-        <v>67</v>
+        <v>219</v>
       </c>
       <c r="R19" t="s">
-        <v>67</v>
+        <v>220</v>
       </c>
       <c r="S19" t="s">
-        <v>67</v>
+        <v>180</v>
       </c>
       <c r="T19" t="s">
         <v>67</v>
@@ -4218,16 +4218,16 @@
         <v>67</v>
       </c>
       <c r="V19" t="s">
-        <v>67</v>
+        <v>221</v>
       </c>
       <c r="W19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="X19" t="s">
-        <v>67</v>
+        <v>222</v>
       </c>
       <c r="Y19" t="s">
-        <v>67</v>
+        <v>221</v>
       </c>
       <c r="Z19" t="s">
         <v>67</v>
@@ -4287,28 +4287,28 @@
         <v>67</v>
       </c>
       <c r="AS19" t="s">
-        <v>67</v>
+        <v>223</v>
       </c>
       <c r="AT19" t="s">
         <v>67</v>
       </c>
       <c r="AU19" t="s">
-        <v>67</v>
+        <v>224</v>
       </c>
       <c r="AV19" t="s">
-        <v>67</v>
+        <v>225</v>
       </c>
       <c r="AW19" t="s">
-        <v>67</v>
+        <v>226</v>
       </c>
       <c r="AX19" t="s">
-        <v>67</v>
+        <v>227</v>
       </c>
       <c r="AY19" t="s">
-        <v>67</v>
+        <v>228</v>
       </c>
       <c r="AZ19" t="s">
-        <v>67</v>
+        <v>229</v>
       </c>
       <c r="BA19" t="s">
         <v>67</v>
@@ -4322,55 +4322,55 @@
         <v>189</v>
       </c>
       <c r="B20" t="s">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="C20" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D20" t="s">
-        <v>115</v>
+        <v>230</v>
       </c>
       <c r="E20" t="s">
-        <v>126</v>
+        <v>231</v>
       </c>
       <c r="F20" t="s">
         <v>71</v>
       </c>
       <c r="G20" t="s">
-        <v>190</v>
+        <v>212</v>
       </c>
       <c r="H20" t="s">
-        <v>191</v>
+        <v>67</v>
       </c>
       <c r="I20" t="s">
-        <v>192</v>
+        <v>232</v>
       </c>
       <c r="J20" t="s">
-        <v>118</v>
+        <v>233</v>
       </c>
       <c r="K20" t="s">
-        <v>193</v>
+        <v>234</v>
       </c>
       <c r="L20" t="s">
         <v>65</v>
       </c>
       <c r="M20" t="s">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="N20" t="s">
-        <v>131</v>
+        <v>236</v>
       </c>
       <c r="O20" t="s">
-        <v>194</v>
+        <v>237</v>
       </c>
       <c r="P20" t="s">
-        <v>195</v>
+        <v>238</v>
       </c>
       <c r="Q20" t="s">
-        <v>196</v>
+        <v>239</v>
       </c>
       <c r="R20" t="s">
-        <v>135</v>
+        <v>220</v>
       </c>
       <c r="S20" t="s">
         <v>180</v>
@@ -4400,10 +4400,10 @@
         <v>67</v>
       </c>
       <c r="AB20" t="s">
-        <v>67</v>
+        <v>240</v>
       </c>
       <c r="AC20" t="s">
-        <v>67</v>
+        <v>241</v>
       </c>
       <c r="AD20" t="s">
         <v>67</v>
@@ -4442,10 +4442,10 @@
         <v>67</v>
       </c>
       <c r="AP20" t="s">
-        <v>67</v>
+        <v>242</v>
       </c>
       <c r="AQ20" t="s">
-        <v>187</v>
+        <v>67</v>
       </c>
       <c r="AR20" t="s">
         <v>67</v>
@@ -4475,7 +4475,7 @@
         <v>67</v>
       </c>
       <c r="BA20" t="s">
-        <v>67</v>
+        <v>243</v>
       </c>
       <c r="BB20" t="s">
         <v>67</v>
@@ -4486,22 +4486,22 @@
         <v>189</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="C21" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D21" t="s">
-        <v>197</v>
+        <v>230</v>
       </c>
       <c r="E21" t="s">
-        <v>126</v>
+        <v>244</v>
       </c>
       <c r="F21" t="s">
-        <v>198</v>
+        <v>71</v>
       </c>
       <c r="G21" t="s">
-        <v>190</v>
+        <v>67</v>
       </c>
       <c r="H21" t="s">
         <v>67</v>
@@ -4510,10 +4510,10 @@
         <v>67</v>
       </c>
       <c r="J21" t="s">
-        <v>199</v>
+        <v>67</v>
       </c>
       <c r="K21" t="s">
-        <v>200</v>
+        <v>67</v>
       </c>
       <c r="L21" t="s">
         <v>67</v>
@@ -4522,25 +4522,25 @@
         <v>67</v>
       </c>
       <c r="N21" t="s">
-        <v>67</v>
+        <v>236</v>
       </c>
       <c r="O21" t="s">
-        <v>201</v>
+        <v>245</v>
       </c>
       <c r="P21" t="s">
-        <v>202</v>
+        <v>67</v>
       </c>
       <c r="Q21" t="s">
-        <v>203</v>
+        <v>67</v>
       </c>
       <c r="R21" t="s">
-        <v>135</v>
+        <v>67</v>
       </c>
       <c r="S21" t="s">
-        <v>180</v>
+        <v>67</v>
       </c>
       <c r="T21" t="s">
-        <v>67</v>
+        <v>246</v>
       </c>
       <c r="U21" t="s">
         <v>67</v>
@@ -4564,7 +4564,7 @@
         <v>67</v>
       </c>
       <c r="AB21" t="s">
-        <v>204</v>
+        <v>67</v>
       </c>
       <c r="AC21" t="s">
         <v>67</v>
@@ -4615,19 +4615,19 @@
         <v>67</v>
       </c>
       <c r="AS21" t="s">
-        <v>205</v>
+        <v>67</v>
       </c>
       <c r="AT21" t="s">
-        <v>206</v>
+        <v>67</v>
       </c>
       <c r="AU21" t="s">
-        <v>207</v>
+        <v>67</v>
       </c>
       <c r="AV21" t="s">
-        <v>208</v>
+        <v>67</v>
       </c>
       <c r="AW21" t="s">
-        <v>209</v>
+        <v>67</v>
       </c>
       <c r="AX21" t="s">
         <v>67</v>
@@ -4646,223 +4646,223 @@
       </c>
     </row>
     <row r="22" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>189</v>
-      </c>
-      <c r="B22" t="s">
-        <v>113</v>
-      </c>
-      <c r="C22" t="s">
-        <v>159</v>
-      </c>
-      <c r="D22" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" t="s">
-        <v>67</v>
-      </c>
-      <c r="F22" t="s">
-        <v>67</v>
-      </c>
-      <c r="G22" t="s">
-        <v>67</v>
-      </c>
-      <c r="H22" t="s">
-        <v>67</v>
-      </c>
-      <c r="I22" t="s">
-        <v>67</v>
-      </c>
-      <c r="J22" t="s">
-        <v>67</v>
-      </c>
-      <c r="K22" t="s">
-        <v>67</v>
-      </c>
-      <c r="L22" t="s">
-        <v>67</v>
-      </c>
-      <c r="M22" t="s">
-        <v>67</v>
-      </c>
-      <c r="N22" t="s">
-        <v>67</v>
-      </c>
-      <c r="O22" t="s">
-        <v>67</v>
-      </c>
-      <c r="P22" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>67</v>
-      </c>
-      <c r="R22" t="s">
-        <v>67</v>
-      </c>
-      <c r="S22" t="s">
-        <v>67</v>
-      </c>
-      <c r="T22" t="s">
-        <v>67</v>
-      </c>
-      <c r="U22" t="s">
-        <v>67</v>
-      </c>
-      <c r="V22" t="s">
-        <v>210</v>
-      </c>
-      <c r="W22" t="s">
-        <v>65</v>
-      </c>
-      <c r="X22" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y22" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY22" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ22" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA22" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB22" t="s">
+      <c r="A22" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="R22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="S22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="T22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="U22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="V22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="W22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="X22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Z22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AC22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AD22" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="AE22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AF22" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="AG22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH22" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="AI22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AJ22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AK22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AM22" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="AN22" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="AO22" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="AP22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AQ22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AR22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AS22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AT22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AU22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AV22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AW22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AX22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AY22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="AZ22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BA22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="BB22" s="2" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="23" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>189</v>
+        <v>247</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>159</v>
+        <v>248</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>211</v>
+        <v>230</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>126</v>
+        <v>249</v>
       </c>
       <c r="F23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>213</v>
-      </c>
       <c r="H23" s="2" t="s">
-        <v>127</v>
+        <v>67</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>72</v>
+        <v>250</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>215</v>
+        <v>251</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>65</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>216</v>
+        <v>235</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="O23" s="2" t="s">
-        <v>218</v>
+        <v>252</v>
       </c>
       <c r="P23" s="2" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="Q23" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="R23" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="S23" s="2" t="s">
         <v>180</v>
@@ -4874,16 +4874,16 @@
         <v>67</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>210</v>
+        <v>255</v>
       </c>
       <c r="W23" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="X23" s="2" t="s">
-        <v>222</v>
+        <v>67</v>
       </c>
       <c r="Y23" s="2" t="s">
-        <v>210</v>
+        <v>255</v>
       </c>
       <c r="Z23" s="2" t="s">
         <v>67</v>
@@ -4943,28 +4943,28 @@
         <v>67</v>
       </c>
       <c r="AS23" s="2" t="s">
-        <v>223</v>
+        <v>67</v>
       </c>
       <c r="AT23" s="2" t="s">
         <v>67</v>
       </c>
       <c r="AU23" s="2" t="s">
-        <v>224</v>
+        <v>67</v>
       </c>
       <c r="AV23" s="2" t="s">
-        <v>225</v>
+        <v>67</v>
       </c>
       <c r="AW23" s="2" t="s">
-        <v>226</v>
+        <v>67</v>
       </c>
       <c r="AX23" s="2" t="s">
-        <v>227</v>
+        <v>67</v>
       </c>
       <c r="AY23" s="2" t="s">
-        <v>228</v>
+        <v>67</v>
       </c>
       <c r="AZ23" s="2" t="s">
-        <v>229</v>
+        <v>67</v>
       </c>
       <c r="BA23" s="2" t="s">
         <v>67</v>
@@ -4975,37 +4975,37 @@
     </row>
     <row r="24" spans="1:54" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>189</v>
+        <v>247</v>
       </c>
       <c r="B24" t="s">
-        <v>125</v>
+        <v>163</v>
       </c>
       <c r="C24" t="s">
-        <v>159</v>
+        <v>248</v>
       </c>
       <c r="D24" t="s">
         <v>230</v>
       </c>
       <c r="E24" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="F24" t="s">
         <v>71</v>
       </c>
       <c r="G24" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H24" t="s">
         <v>67</v>
       </c>
       <c r="I24" t="s">
-        <v>232</v>
+        <v>256</v>
       </c>
       <c r="J24" t="s">
         <v>233</v>
       </c>
       <c r="K24" t="s">
-        <v>234</v>
+        <v>257</v>
       </c>
       <c r="L24" t="s">
         <v>65</v>
@@ -5017,16 +5017,16 @@
         <v>236</v>
       </c>
       <c r="O24" t="s">
-        <v>237</v>
+        <v>66</v>
       </c>
       <c r="P24" t="s">
-        <v>238</v>
+        <v>258</v>
       </c>
       <c r="Q24" t="s">
-        <v>239</v>
+        <v>259</v>
       </c>
       <c r="R24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="S24" t="s">
         <v>180</v>
@@ -5056,10 +5056,10 @@
         <v>67</v>
       </c>
       <c r="AB24" t="s">
-        <v>240</v>
+        <v>67</v>
       </c>
       <c r="AC24" t="s">
-        <v>241</v>
+        <v>67</v>
       </c>
       <c r="AD24" t="s">
         <v>67</v>
@@ -5098,7 +5098,7 @@
         <v>67</v>
       </c>
       <c r="AP24" t="s">
-        <v>242</v>
+        <v>67</v>
       </c>
       <c r="AQ24" t="s">
         <v>67</v>
@@ -5131,829 +5131,9 @@
         <v>67</v>
       </c>
       <c r="BA24" t="s">
-        <v>243</v>
+        <v>67</v>
       </c>
       <c r="BB24" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="25" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>189</v>
-      </c>
-      <c r="B25" t="s">
-        <v>138</v>
-      </c>
-      <c r="C25" t="s">
-        <v>159</v>
-      </c>
-      <c r="D25" t="s">
-        <v>230</v>
-      </c>
-      <c r="E25" t="s">
-        <v>244</v>
-      </c>
-      <c r="F25" t="s">
-        <v>71</v>
-      </c>
-      <c r="G25" t="s">
-        <v>67</v>
-      </c>
-      <c r="H25" t="s">
-        <v>67</v>
-      </c>
-      <c r="I25" t="s">
-        <v>67</v>
-      </c>
-      <c r="J25" t="s">
-        <v>67</v>
-      </c>
-      <c r="K25" t="s">
-        <v>67</v>
-      </c>
-      <c r="L25" t="s">
-        <v>67</v>
-      </c>
-      <c r="M25" t="s">
-        <v>67</v>
-      </c>
-      <c r="N25" t="s">
-        <v>236</v>
-      </c>
-      <c r="O25" t="s">
-        <v>245</v>
-      </c>
-      <c r="P25" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>67</v>
-      </c>
-      <c r="R25" t="s">
-        <v>67</v>
-      </c>
-      <c r="S25" t="s">
-        <v>67</v>
-      </c>
-      <c r="T25" t="s">
-        <v>246</v>
-      </c>
-      <c r="U25" t="s">
-        <v>67</v>
-      </c>
-      <c r="V25" t="s">
-        <v>67</v>
-      </c>
-      <c r="W25" t="s">
-        <v>67</v>
-      </c>
-      <c r="X25" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y25" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY25" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ25" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA25" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB25" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="26" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A26" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="O26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="P26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="S26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="W26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="X26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD26" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="AE26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF26" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="AG26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH26" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="AI26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM26" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="AN26" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="AO26" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="AP26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA26" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB26" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="27" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A27" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="O27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="P27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="R27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="S27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="T27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V27" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="W27" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="X27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA27" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB27" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="O28" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="P28" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="Q28" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="R28" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="S28" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="T28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="U28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="V28" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="W28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="X28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y28" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="Z28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA28" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB28" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="29" spans="1:54" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>247</v>
-      </c>
-      <c r="B29" t="s">
-        <v>164</v>
-      </c>
-      <c r="C29" t="s">
-        <v>248</v>
-      </c>
-      <c r="D29" t="s">
-        <v>230</v>
-      </c>
-      <c r="E29" t="s">
-        <v>250</v>
-      </c>
-      <c r="F29" t="s">
-        <v>71</v>
-      </c>
-      <c r="G29" t="s">
-        <v>213</v>
-      </c>
-      <c r="H29" t="s">
-        <v>67</v>
-      </c>
-      <c r="I29" t="s">
-        <v>256</v>
-      </c>
-      <c r="J29" t="s">
-        <v>233</v>
-      </c>
-      <c r="K29" t="s">
-        <v>257</v>
-      </c>
-      <c r="L29" t="s">
-        <v>65</v>
-      </c>
-      <c r="M29" t="s">
-        <v>235</v>
-      </c>
-      <c r="N29" t="s">
-        <v>236</v>
-      </c>
-      <c r="O29" t="s">
-        <v>66</v>
-      </c>
-      <c r="P29" t="s">
-        <v>258</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>259</v>
-      </c>
-      <c r="R29" t="s">
-        <v>221</v>
-      </c>
-      <c r="S29" t="s">
-        <v>180</v>
-      </c>
-      <c r="T29" t="s">
-        <v>67</v>
-      </c>
-      <c r="U29" t="s">
-        <v>67</v>
-      </c>
-      <c r="V29" t="s">
-        <v>67</v>
-      </c>
-      <c r="W29" t="s">
-        <v>67</v>
-      </c>
-      <c r="X29" t="s">
-        <v>67</v>
-      </c>
-      <c r="Y29" t="s">
-        <v>67</v>
-      </c>
-      <c r="Z29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AB29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AC29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AD29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AE29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AF29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AG29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AH29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AI29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AK29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AL29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AM29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AN29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AO29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AP29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AQ29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AR29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AS29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AT29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AU29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AV29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AW29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AX29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AY29" t="s">
-        <v>67</v>
-      </c>
-      <c r="AZ29" t="s">
-        <v>67</v>
-      </c>
-      <c r="BA29" t="s">
-        <v>67</v>
-      </c>
-      <c r="BB29" t="s">
         <v>260</v>
       </c>
     </row>

</xml_diff>